<commit_message>
feat: deep sub-categorization of courses across 13 tracks and 224 curated tools
</commit_message>
<xml_diff>
--- a/📊 Websites_Master_List.xlsx
+++ b/📊 Websites_Master_List.xlsx
@@ -1204,7 +1204,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Excel: ⬇️ Video Downloaders.xlsx (URL Trick 3)</t>
+          <t>Excel: ⬇️ Video Downloaders.xlsx</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Facebook Video Downloader</t>
+          <t>Online downloader for Facebook videos, clips, and private videos.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Facebook Video Downloader</t>
+          <t>Fast online Facebook Video Downloader for MP4 and HD videos.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Instagram Downloader</t>
+          <t>Download Instagram photos, videos, reels, IGTV, and carousels online.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Excel: ⬇️ Video Downloaders.xlsx (URL Trick 2)</t>
+          <t>Excel: ⬇️ Video Downloaders.xlsx</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Pinterest Video Downloader</t>
+          <t>Fast Pinterest video, GIF, and photo downloader.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Subtitle Automation Tool</t>
+          <t>Automated open-source subtitle generator and downloader tool.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Twitter Video Downloader</t>
+          <t>Direct Twitter (X) video and GIF downloader online.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Universal Media Downloader</t>
+          <t>Universal media downloader for YouTube, Twitter, Instagram, Reddit with zero ads.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: YouTube to MP4 Converter</t>
+          <t>Convert and download YouTube videos to MP4 high-speed online.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Excel: ⬇️ Video Downloaders.xlsx (URL Trick 1)</t>
+          <t>Excel: ⬇️ Video Downloaders.xlsx</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>YouTube Video , Mp3 download with timestamp</t>
+          <t>YouTube Video &amp; MP3 Timestamp Downloader</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: YouTube Video , Mp3 download with timestamp</t>
+          <t>Tool and tutorial to download specific timestamp clips from YouTube videos as MP3 or MP4.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: YouTube Video Downloader</t>
+          <t>Online YouTube video downloader for 1080p, 720p, and MP3 audio.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="G156" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: File Search Engine</t>
+          <t>Open file and media search engine indexing millions of web files.</t>
         </is>
       </c>
       <c r="H156" s="4" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="G160" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Image Processing Tool</t>
+          <t>Online image compressor, resizer, and converter tool.</t>
         </is>
       </c>
       <c r="H160" s="4" t="inlineStr">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Facebook Video Downloader</t>
+          <t>Online downloader for Facebook videos, clips, and private videos.</t>
         </is>
       </c>
     </row>
@@ -11932,7 +11932,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Facebook Video Downloader</t>
+          <t>Fast online Facebook Video Downloader for MP4 and HD videos.</t>
         </is>
       </c>
     </row>
@@ -11962,7 +11962,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Instagram Downloader</t>
+          <t>Download Instagram photos, videos, reels, IGTV, and carousels online.</t>
         </is>
       </c>
     </row>
@@ -12022,7 +12022,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Pinterest Video Downloader</t>
+          <t>Fast Pinterest video, GIF, and photo downloader.</t>
         </is>
       </c>
     </row>
@@ -12052,7 +12052,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Subtitle Automation Tool</t>
+          <t>Automated open-source subtitle generator and downloader tool.</t>
         </is>
       </c>
     </row>
@@ -12082,7 +12082,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Twitter Video Downloader</t>
+          <t>Direct Twitter (X) video and GIF downloader online.</t>
         </is>
       </c>
     </row>
@@ -12112,7 +12112,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Universal Media Downloader</t>
+          <t>Universal media downloader for YouTube, Twitter, Instagram, Reddit with zero ads.</t>
         </is>
       </c>
     </row>
@@ -12142,7 +12142,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: YouTube to MP4 Converter</t>
+          <t>Convert and download YouTube videos to MP4 high-speed online.</t>
         </is>
       </c>
     </row>
@@ -12187,7 +12187,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>YouTube Video , Mp3 download with timestamp</t>
+          <t>YouTube Video &amp; MP3 Timestamp Downloader</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -12202,7 +12202,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: YouTube Video , Mp3 download with timestamp</t>
+          <t>Tool and tutorial to download specific timestamp clips from YouTube videos as MP3 or MP4.</t>
         </is>
       </c>
     </row>
@@ -12232,7 +12232,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: YouTube Video Downloader</t>
+          <t>Online YouTube video downloader for 1080p, 720p, and MP3 audio.</t>
         </is>
       </c>
     </row>
@@ -13124,15 +13124,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13143,25 +13144,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Website Name</t>
+          <t>Course / Platform Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Track / Sub-Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Website Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Official URL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Pricing</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -13178,20 +13184,25 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
+          <t>🧠 Agentic AI &amp; Autonomous Systems</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
           <t>Agentic AI Course</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/a-b-c-of-coding-to-build-ai-agents</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: A B C of Coding to Build AI Agents (Agentic AI Course)</t>
         </is>
@@ -13208,20 +13219,25 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
+          <t>🧠 Agentic AI &amp; Autonomous Systems</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
           <t>Agentic AI Course</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/agentic-ai-design-pattern</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Agentic : AI Design Pattern (Agentic AI Course)</t>
         </is>
@@ -13238,20 +13254,25 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t>🧠 Agentic AI &amp; Autonomous Systems</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
           <t>Agentic AI Course</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/build-a-resume-review-agentic-system-with-crewai</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Build a Resume Review Agentic System with CrewAI (Agentic AI Course)</t>
         </is>
@@ -13268,20 +13289,25 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>🧠 Agentic AI &amp; Autonomous Systems</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>Agentic AI Course</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/building-agentic-ai-system-with-with-bedrock</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Building Agentic AI System with Bedrock (Agentic AI Course)</t>
         </is>
@@ -13298,20 +13324,25 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
+          <t>🧠 Agentic AI &amp; Autonomous Systems</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
           <t>Agentic AI Course</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/knowledge-bases-and-memory-for-agentic-ai</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Knowledge Bases &amp; Memory for Agentic AI (Agentic AI Course)</t>
         </is>
@@ -13328,20 +13359,25 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
           <t>AI Course Platform</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>https://www.elementsofai.com</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Elements of AI (AI Course Platform)</t>
         </is>
@@ -13358,20 +13394,25 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>🔬 Frontier AI Models Deep Dive</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
           <t>AI Model Deep Dive Course</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/deep-dive-into-qwq-32b</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Deep Dive Into QwQ-32B (AI Model Deep Dive Course)</t>
         </is>
@@ -13388,20 +13429,25 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>🔬 Frontier AI Models Deep Dive</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
           <t>AI Model Deep Dive Course</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/exploring-openai-o3-and-o4-mini</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Exploring OpenAI o3 and o4-mini (AI Model Deep Dive Course)</t>
         </is>
@@ -13418,20 +13464,25 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>🔬 Frontier AI Models Deep Dive</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
           <t>AI Model Deep Dive Course</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/getting-started-with-deepseek</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Getting Started with DeepSeek-AI (AI Model Deep Dive Course)</t>
         </is>
@@ -13448,20 +13499,25 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
+          <t>🔬 Frontier AI Models Deep Dive</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
           <t>AI Model Deep Dive Course</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/getting-started-with-openai-o3-mini</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Getting Started with OpenAI o3-mini (AI Model Deep Dive Course)</t>
         </is>
@@ -13478,20 +13534,25 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
+          <t>🔬 Frontier AI Models Deep Dive</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
           <t>AI Model Deep Dive Course</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/xai-grok-3-smartest-ai-on-earth</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: xAI Grok 3: Smartest AI on Earth (AI Model Deep Dive Course)</t>
         </is>
@@ -13508,20 +13569,25 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
           <t>AI Training Course</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>https://www.databricks.com/learn/training/generative-ai-fundamentals</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Databricks – Generative AI Fundamentals (AI Training Course)</t>
         </is>
@@ -13538,20 +13604,25 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>☁️ Cloud Computing &amp; Google Skills</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
           <t>Cloud Training Path</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>https://www.cloudskillsboost.google/paths/118</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Free + Paid</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Google Cloud Skills Boost (Cloud Training Path)</t>
         </is>
@@ -13568,20 +13639,25 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>💻 Computer Education &amp; Web Development</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
           <t>Computer Courses Platform</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>https://www.stpcomputereducation.com/courses</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Free + Paid</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: STP Computer Education – Courses (Computer Courses Platform)</t>
         </is>
@@ -13598,20 +13674,25 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>https://chemequations.com</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Auto-balance chemical equations instantly - essential tool for chemistry homework and learning</t>
         </is>
@@ -13628,20 +13709,25 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>https://classcentral.com</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Search engine aggregating online courses from all major platforms with reviews and ratings</t>
         </is>
@@ -13658,20 +13744,25 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>https://cymath.com</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Freemium</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Step-by-step math problem solver that shows you how to get the answer</t>
         </is>
@@ -13688,20 +13779,25 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>https://dungeonscrawl.com</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Freemium</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Create custom dungeon maps online for tabletop RPGs and virtual tabletop sessions</t>
         </is>
@@ -13718,20 +13814,25 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>https://human.biodigital.com</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Interactive 3D human anatomy model for medical students and curious minds to explore</t>
         </is>
@@ -13748,20 +13849,25 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>https://kiddoworksheets.com</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Free printable worksheets for kids covering math reading and educational activities</t>
         </is>
@@ -13778,20 +13884,25 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>https://litsolutions.org</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Free textbook solutions and homework help with step-by-step workings for STEM courses</t>
         </is>
@@ -13808,20 +13919,25 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>https://mindluster.com</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>Free online courses with certificates you can add to your resume upon completion</t>
         </is>
@@ -13838,20 +13954,25 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>https://musicca.com</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Interactive music theory lessons with virtual instruments and exercises to practice concepts</t>
         </is>
@@ -13868,20 +13989,25 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>https://phet.colorado.edu</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>Free interactive science simulations from University of Colorado for physics chemistry and biology</t>
         </is>
@@ -13898,20 +14024,25 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>https://smart.servier.com</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>Free high-resolution medical and scientific images for anatomy biology and healthcare projects</t>
         </is>
@@ -13928,20 +14059,25 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>https://spacetypegenerator.com</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>Animated typography effects generator for creating dynamic text for videos and social media</t>
         </is>
@@ -13958,20 +14094,25 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>https://typelit.io</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Freemium</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>Practice typing by retyping classic literature - combine skill development with reading great books</t>
         </is>
@@ -13988,20 +14129,25 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>https://typingclub.com</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Freemium</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>Structured typing lessons for schools and individuals with gamified progress tracking</t>
         </is>
@@ -14018,20 +14164,25 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>https://wolframalpha.com</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Freemium</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>Computational knowledge engine that answers questions with computed data rather than web links</t>
         </is>
@@ -14048,20 +14199,25 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
           <t>Educational Learning Platform</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>https://zty.pe</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>Typing game where you shoot down enemy ships by typing words - fun skill practice</t>
         </is>
@@ -14078,20 +14234,25 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
+          <t>🗣️ English &amp; Language Learning</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
           <t>English Learning Page</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>https://www.instagram.com/learn_english_with_shaba</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Instagram – Learn English With Shaba (English Learning Page)</t>
         </is>
@@ -14108,20 +14269,25 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
+          <t>🗣️ English &amp; Language Learning</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
           <t>English Learning Video</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>https://youtu.be/ES4TpVsTkgc</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: YouTube – dLKPBSov2F4 (English Learning Video)</t>
         </is>
@@ -14138,20 +14304,25 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
+          <t>🎁 Free Program Combos &amp; Bundles</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
           <t>Free Program Combo Bundle</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/learning-path/data-science-program</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Data Science Free Program - 9 Courses Combo (Free Program Combo Bundle)</t>
         </is>
@@ -14168,20 +14339,25 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
+          <t>🎁 Free Program Combos &amp; Bundles</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
           <t>Free Program Combo Bundle</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/learning-path/generative-ai-program-free</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: GenAI Free Program - 7 Courses Combo (Free Program Combo Bundle)</t>
         </is>
@@ -14198,20 +14374,25 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
+          <t>📈 Data Analytics, SQL &amp; Fundamental Tech</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
           <t>Fundamental Tech Course</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/essential-sql-skills-for-data-beginners</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Essential : SQL Skills for Data Beginners (Fundamental Tech Course)</t>
         </is>
@@ -14228,20 +14409,25 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
+          <t>📈 Data Analytics, SQL &amp; Fundamental Tech</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
           <t>Fundamental Tech Course</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/excel-from-beginner-to-expert</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Excel : From Beginner to Expert (Fundamental Tech Course)</t>
         </is>
@@ -14258,20 +14444,25 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
+          <t>📈 Data Analytics, SQL &amp; Fundamental Tech</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
           <t>Fundamental Tech Course</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/genai-landscape</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: GenAI for Everyone (Fundamental Tech Course)</t>
         </is>
@@ -14288,20 +14479,25 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
+          <t>📈 Data Analytics, SQL &amp; Fundamental Tech</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
           <t>Fundamental Tech Course</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/getting-started-with-tableau</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Getting Started with Tableau (Fundamental Tech Course)</t>
         </is>
@@ -14318,20 +14514,25 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
+          <t>📈 Data Analytics, SQL &amp; Fundamental Tech</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
           <t>Fundamental Tech Course</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/introduction-to-data-science</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Introduction to Python (Fundamental Tech Course)</t>
         </is>
@@ -14348,20 +14549,25 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
           <t>Generative AI Course</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/build-product-10x-faster-with-genai</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Build Products 10x Faster with GenAI (Generative AI Course)</t>
         </is>
@@ -14378,20 +14584,25 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
           <t>Generative AI Course</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/deepseek-from-scratch</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: DeepSeek from Scratch (Generative AI Course)</t>
         </is>
@@ -14408,20 +14619,25 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
           <t>Generative AI Course</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/genai-applied-to-quantitative-finance-for-control-implementation</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: GenAI for Quantitative Finance &amp; Control Implementation (Generative AI Course)</t>
         </is>
@@ -14438,20 +14654,25 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
           <t>Generative AI Course</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/genai-a-way-of-life</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Generative AI - A Way of Life (Generative AI Course)</t>
         </is>
@@ -14468,20 +14689,25 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
           <t>Generative AI Course</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/reimagining-genai-common-mistakes-and-best-practices-for-success</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Reimagining GenAI: Common Mistakes and Best Practices for Success (Generative AI Course)</t>
         </is>
@@ -14498,20 +14724,25 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/a-complete-mlops-journey</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: A Complete MLops Journey (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14528,20 +14759,25 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/a-comprehensive-learning-path-to-become-a-data-scientist-in-twenty-twenty-four</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: A Comprehensive Learning Path to Become a Data Scientist in 2025 (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14558,20 +14794,25 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/bagging-boosting-ML-Algorithms</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Bagging and Boosting ML Algorithms (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14588,20 +14829,25 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/free-building-textclassification-natural-language-processing</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Building Text Classification Models in NLP (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14618,20 +14864,25 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/dimensionality-reduction-for-machine-learning</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Dimensionality Reduction for Machine Learning (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14648,20 +14899,25 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/ensemble-learning-and-ensemble-learning-techniques</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Ensemble Learning and Ensemble Learning Techniques (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14678,20 +14934,25 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/Fundamentals-of-Regression-Analysis</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Fundamentals of Regression Analysis (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14708,20 +14969,25 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/getting-started-with-deep-learning</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Getting Started with Deep Learning (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14738,20 +15004,25 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/getting-started-with-llms</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Getting Started With Large Language Models (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14768,20 +15039,25 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/introduction-to-ai-ml</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Introduction to AI &amp; ML (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14798,20 +15074,25 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/introduction-to-transformers-and-attention-mechanisms</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Introduction to Transformers and Attention Mechanisms (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14828,20 +15109,25 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/K-Nearest-Neighbors-KNN-Algorithm</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: K-Nearest Neighbors (KNN) Algorithm in Python and R (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14858,20 +15144,25 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/machine-learning-certification-program-beginners</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Machine Learning Certification course for Beginners (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14888,20 +15179,25 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/naive-bayes</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Naive Bayes from Scratch (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14918,20 +15214,25 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/free-unsupervised-ml-guide</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: The A to Z of Unsupervised ML (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14948,20 +15249,25 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/free-understanding-linear-regression</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Understanding Linear Regression (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -14978,20 +15284,25 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
           <t>Machine Learning &amp; Deep Learning Course</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/understanding-the-working-of-neural-networks</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F62" s="4" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Understanding the working of Neural Networks (Machine Learning &amp; Deep Learning Course)</t>
         </is>
@@ -15008,20 +15319,25 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
+          <t>☁️ Cloud Computing &amp; Google Skills</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
           <t>Official Google Training</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>https://skillshop.withgoogle.com</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Google Skillshop (Official Google Training)</t>
         </is>
@@ -15038,20 +15354,25 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
           <t>Online Course</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>https://www.coursera.org/learn/generative-ai-for-everyone</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>Free + Paid</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Coursera – Generative AI for Everyone (Online Course)</t>
         </is>
@@ -15068,20 +15389,25 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
           <t>Online Course</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>https://www.coursera.org/learn/generative-ai-with-llms</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>Free + Paid</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr">
+      <c r="G65" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Coursera – Generative AI with LLMs (Online Course)</t>
         </is>
@@ -15098,20 +15424,25 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
+          <t>📊 Machine Learning &amp; Deep Learning Mastery</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
           <t>Online Course</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>https://www.coursera.org/learn/machine-learning</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Free + Paid</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Coursera – Machine Learning (Online Course)</t>
         </is>
@@ -15128,20 +15459,25 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
+          <t>📈 Data Analytics, SQL &amp; Fundamental Tech</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
           <t>Online Course Platform</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="E67" s="5" t="inlineStr">
         <is>
           <t>https://www.mygreatlearning.com/academy</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Great Learning Academy (Online Course Platform)</t>
         </is>
@@ -15158,20 +15494,25 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
+          <t>🤖 Generative AI &amp; LLM Engineering</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
           <t>Open Source AI Course</t>
         </is>
       </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="E68" s="5" t="inlineStr">
         <is>
           <t>https://github.com/microsoft/generative-ai-for-beginners</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: GitHub – Microsoft Generative AI for Beginners (Open Source AI Course)</t>
         </is>
@@ -15188,20 +15529,25 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
+          <t>📈 Data Analytics, SQL &amp; Fundamental Tech</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
           <t>Professional Certificate</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="E69" s="5" t="inlineStr">
         <is>
           <t>https://www.coursera.org/professional-certificates/google-data-analytics</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: Coursera – Google Data Analytics (Professional Certificate)</t>
         </is>
@@ -15218,20 +15564,25 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D70" s="5" t="inlineStr">
+      <c r="E70" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/big-mart-sales-prediction-using-r</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Big Mart Sales Prediction Using R (Project-Based Learning Course)</t>
         </is>
@@ -15248,20 +15599,25 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="E71" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/build-data-pipelines-with-apache-airflow</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Build Data Pipelines with Apache Airflow (Project-Based Learning Course)</t>
         </is>
@@ -15278,20 +15634,25 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/building-a-deep-research-ai-agent</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Building a Deep Research AI Agent (Project-Based Learning Course)</t>
         </is>
@@ -15308,20 +15669,25 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/coding-a-chatgpt-style-language-model-from-scratch-in-pytorch</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Coding a ChatGPT-style Language Model From Scratch in Pytorch (Project-Based Learning Course)</t>
         </is>
@@ -15338,20 +15704,25 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D74" s="5" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/how-to-build-an-image-generator-web-app-with-zero-coding</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: How to Build an Image Generator Web App with Zero Coding (Project-Based Learning Course)</t>
         </is>
@@ -15368,20 +15739,25 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="E75" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/loan-prediction-practice-problem-using-python</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Loan Prediction Practice Problem (Using Python) (Project-Based Learning Course)</t>
         </is>
@@ -15398,20 +15774,25 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D76" s="5" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/model-deployment-using-fastapi</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Model Deployment using FastAPI (Project-Based Learning Course)</t>
         </is>
@@ -15428,20 +15809,25 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
+          <t>🛠️ Project-Based AI &amp; Data Pipelines</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
           <t>Project-Based Learning Course</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
+      <c r="E77" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/openengage-a-complete-ai-driven-marketing-engine</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: OpenEngage: Build a complete AI Driven Marketing Engine (Project-Based Learning Course)</t>
         </is>
@@ -15458,20 +15844,25 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
+          <t>🔗 RAG (Retrieval-Augmented Generation)</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
           <t>RAG Application Course</t>
         </is>
       </c>
-      <c r="D78" s="5" t="inlineStr">
+      <c r="E78" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/build-a-document-retriever-search-engine-with-langchain</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Build a Document Retriever Search Engine with LangChain (RAG Application Course)</t>
         </is>
@@ -15488,20 +15879,25 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
+          <t>🔗 RAG (Retrieval-Augmented Generation)</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
           <t>RAG Application Course</t>
         </is>
       </c>
-      <c r="D79" s="5" t="inlineStr">
+      <c r="E79" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/building-first-rag-systems-using-llamaindex</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Build your first RAG system using Llamaindex (RAG Application Course)</t>
         </is>
@@ -15518,20 +15914,25 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
+          <t>🔗 RAG (Retrieval-Augmented Generation)</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
           <t>RAG Application Course</t>
         </is>
       </c>
-      <c r="D80" s="5" t="inlineStr">
+      <c r="E80" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/end-to-end-app-rag-application-development-with-langchain-and-streamlit</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: End to end RAG Application Development with LangChain and Streamlit (RAG Application Course)</t>
         </is>
@@ -15548,20 +15949,25 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
+          <t>🔗 RAG (Retrieval-Augmented Generation)</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
           <t>RAG Application Course</t>
         </is>
       </c>
-      <c r="D81" s="5" t="inlineStr">
+      <c r="E81" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/improving-real-world-rag-systems-key-challenges</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Improving Real World RAG Systems :Key Challenges (RAG Application Course)</t>
         </is>
@@ -15578,20 +15984,25 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
+          <t>🔗 RAG (Retrieval-Augmented Generation)</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
           <t>RAG Application Course</t>
         </is>
       </c>
-      <c r="D82" s="5" t="inlineStr">
+      <c r="E82" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/mastering-multimodal-rag-and-embeddings-with-amazon-nova-and-bedrock</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F82" s="4" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Mastering Multimodal RAG &amp; Embeddings with Amazon Nova &amp; Bedrock (RAG Application Course)</t>
         </is>
@@ -15608,20 +16019,25 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
+          <t>🌐 Academic STEM Tools &amp; Learning Platforms</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
           <t>Skill Development Platform</t>
         </is>
       </c>
-      <c r="D83" s="5" t="inlineStr">
+      <c r="E83" s="5" t="inlineStr">
         <is>
           <t>https://www.learnvern.com</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>Free + Paid</t>
         </is>
       </c>
-      <c r="F83" s="4" t="inlineStr">
+      <c r="G83" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: LearnVern (Skill Development Platform)</t>
         </is>
@@ -15638,20 +16054,25 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
+          <t>💻 Computer Education &amp; Web Development</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
           <t>Study Notes / Learning Material</t>
         </is>
       </c>
-      <c r="D84" s="5" t="inlineStr">
+      <c r="E84" s="5" t="inlineStr">
         <is>
           <t>https://www.stpcomputereducation.com/notes</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F84" s="4" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: STP Computer Education – Notes (Study Notes / Learning Material)</t>
         </is>
@@ -15668,20 +16089,25 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
+          <t>⚡ Vibe Coding &amp; AI Automation</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
           <t>Vibe Coding Course</t>
         </is>
       </c>
-      <c r="D85" s="5" t="inlineStr">
+      <c r="E85" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/building-a-customized-newsletter-ai-agent</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Building a Customized Newsletter AI Agent (Vibe Coding Course)</t>
         </is>
@@ -15698,20 +16124,25 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
+          <t>⚡ Vibe Coding &amp; AI Automation</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
           <t>Vibe Coding Course</t>
         </is>
       </c>
-      <c r="D86" s="5" t="inlineStr">
+      <c r="E86" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/guide-to-vibe-coding-in-windsurf</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F86" s="4" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Guide to Vibe Coding in Windsurf (Vibe Coding Course)</t>
         </is>
@@ -15728,20 +16159,25 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
+          <t>⚡ Vibe Coding &amp; AI Automation</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
           <t>Vibe Coding Course</t>
         </is>
       </c>
-      <c r="D87" s="5" t="inlineStr">
+      <c r="E87" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/n8n-a-complete-guide-to-the-automation-tool</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F87" s="4" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: n8n - A Complete Guide to Automation Tool (Vibe Coding Course)</t>
         </is>
@@ -15758,20 +16194,25 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
+          <t>⚡ Vibe Coding &amp; AI Automation</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
           <t>Vibe Coding Course</t>
         </is>
       </c>
-      <c r="D88" s="5" t="inlineStr">
+      <c r="E88" s="5" t="inlineStr">
         <is>
           <t>https://www.analyticsvidhya.com/courses/vibe-coding-with-replit</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F88" s="4" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
         <is>
           <t>Comprehensive free training course: Vibe Coding with Replit (Vibe Coding Course)</t>
         </is>
@@ -15788,20 +16229,25 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
+          <t>💻 Computer Education &amp; Web Development</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
           <t>Web Development Course</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
+      <c r="E89" s="5" t="inlineStr">
         <is>
           <t>https://www.stpcomputereducation.com/courses/web-development.html</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>Free + Paid</t>
         </is>
       </c>
-      <c r="F89" s="4" t="inlineStr">
+      <c r="G89" s="4" t="inlineStr">
         <is>
           <t>Free education and certified training: STP Computer Education – Web Development (Web Development Course)</t>
         </is>
@@ -15809,94 +16255,94 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16366,7 +16812,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: File Search Engine</t>
+          <t>Open file and media search engine indexing millions of web files.</t>
         </is>
       </c>
     </row>
@@ -16486,7 +16932,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>High-speed online tool: Image Processing Tool</t>
+          <t>Online image compressor, resizer, and converter tool.</t>
         </is>
       </c>
     </row>

</xml_diff>